<commit_message>
Verify E3 against Beyond Connections (2015); correct MTF capacity wording; rebuild register, workbooks and book
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192koLK9F8fRH5Bfqszi1tY
</commit_message>
<xml_diff>
--- a/output/04_SOURCE_REGISTER_v1.0.xlsx
+++ b/output/04_SOURCE_REGISTER_v1.0.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy_Map" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Register'!$A$1:$T$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Register'!$A$1:$T$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -680,7 +680,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18">
@@ -724,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T70"/>
+  <dimension ref="A1:T72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4642,86 +4642,94 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>E3-01</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Multi-Tier Framework capacity thresholds (T4 at least 800 W / 3.4 kWh a day; T5 at least 2 kW / 8.2 kWh a day)</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Multi-Tier Framework household electricity supply, capacity: Tier 1 min 3 W or 12 Wh a day; Tier 2 min 50 W or 200 Wh; Tier 3 min 200 W or 1.0 kWh; Tier 4 min 800 W or 3.4 kWh; Tier 5 min 2 kW or 8.2 kWh</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
         <is>
           <t>T1-T5</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="9" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>Beyond Connections: Energy Access Redefined</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Beyond Connections: Energy Access Redefined (Technical Report 008/15, conceptualization report)</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
         <is>
           <t>ESMAP / World Bank</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>2015</t>
-        </is>
-      </c>
-      <c r="I45" s="7" t="inlineStr">
-        <is>
-          <t>Not held</t>
-        </is>
-      </c>
-      <c r="J45" s="7" t="inlineStr">
-        <is>
-          <t>PAGE TO VERIFY</t>
-        </is>
-      </c>
-      <c r="K45" s="7" t="inlineStr"/>
-      <c r="L45" s="7" t="inlineStr"/>
-      <c r="M45" s="7" t="inlineStr">
-        <is>
-          <t>Thresholds recorded from earlier research; framework report not read</t>
-        </is>
-      </c>
-      <c r="N45" s="7" t="inlineStr">
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>July 2015</t>
+        </is>
+      </c>
+      <c r="I45" s="9" t="inlineStr">
+        <is>
+          <t>BEYOND CONNECTIONS  Energy Access Redefined.pdf (244 pages; author's Google Drive, SHA-256 9d23881a...c1d26b)</t>
+        </is>
+      </c>
+      <c r="J45" s="9" t="inlineStr">
+        <is>
+          <t>20 (report page 6)</t>
+        </is>
+      </c>
+      <c r="K45" s="9" t="inlineStr">
+        <is>
+          <t>Table ES.1, Multi-tier Matrix for Measuring Access to Household Electricity Supply</t>
+        </is>
+      </c>
+      <c r="L45" s="9" t="inlineStr">
+        <is>
+          <t>Project file (retrieved from the author's Drive, 4 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>Read in the document</t>
+        </is>
+      </c>
+      <c r="N45" s="9" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="O45" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
-        </is>
-      </c>
-      <c r="P45" s="7" t="inlineStr">
+      <c r="O45" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P45" s="9" t="inlineStr">
         <is>
           <t>Ch 2.6</t>
         </is>
       </c>
-      <c r="Q45" s="7" t="inlineStr">
-        <is>
-          <t>Products tier labels</t>
-        </is>
-      </c>
-      <c r="R45" s="7" t="inlineStr"/>
-      <c r="S45" s="7" t="inlineStr"/>
-      <c r="T45" s="7" t="inlineStr">
+      <c r="Q45" s="9" t="inlineStr">
+        <is>
+          <t>Products tier labels (capacity attribute only)</t>
+        </is>
+      </c>
+      <c r="R45" s="9" t="inlineStr"/>
+      <c r="S45" s="9" t="inlineStr"/>
+      <c r="T45" s="9" t="inlineStr">
         <is>
           <t>SR20</t>
         </is>
@@ -4730,70 +4738,72 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>E4-01</t>
+          <t>E3-02</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>M-KOPA UK LIMITED revenue (sales of carbon credits)</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="n">
-        <v>1712776</v>
+          <t>Household electricity attributes are capacity, duration (daily and evening supply), reliability, quality, affordability, legality, and health and safety; the lowest tier among all attributes determines the household's overall tier</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>FY2024 (FY2023: 718,100)</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>M-KOPA UK LIMITED, Annual Report and Accounts, year ended 31 December 2024</t>
+          <t>Beyond Connections: Energy Access Redefined (Technical Report 008/15, conceptualization report)</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>Companies House (company 10229661)</t>
+          <t>ESMAP / World Bank</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>Approved 20 Jun 2025; filed 25 Sep 2025</t>
+          <t>July 2015</t>
         </is>
       </c>
       <c r="I46" s="9" t="inlineStr">
         <is>
-          <t>245b3bf6-companies_house_document.pdf (34 pages, scanned)</t>
+          <t>BEYOND CONNECTIONS  Energy Access Redefined.pdf (244 pages; author's Google Drive, SHA-256 9d23881a...c1d26b)</t>
         </is>
       </c>
       <c r="J46" s="9" t="inlineStr">
         <is>
-          <t>10 (filing page 8); 18 (filing page 16, note 2.1)</t>
+          <t>19 (report page 5)</t>
         </is>
       </c>
       <c r="K46" s="9" t="inlineStr">
         <is>
-          <t>Statement of profit or loss; note 2.1 Sale of carbon credits</t>
+          <t>Executive Summary</t>
         </is>
       </c>
       <c r="L46" s="9" t="inlineStr">
         <is>
-          <t>Project file (uploaded 3 Oct 2026)</t>
+          <t>Project file (retrieved from the author's Drive, 4 Oct 2026)</t>
         </is>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>Audited statutory accounts (auditor KLSA LLP), read page by page</t>
+          <t>Read in the document</t>
         </is>
       </c>
       <c r="N46" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O46" s="9" t="inlineStr">
@@ -4803,89 +4813,87 @@
       </c>
       <c r="P46" s="9" t="inlineStr">
         <is>
-          <t>Planned: Ch 15 (as an illustration of entity checking)</t>
+          <t>Ch 2.6</t>
         </is>
       </c>
       <c r="Q46" s="9" t="inlineStr">
         <is>
-          <t>Not used: different entity and activity; not a PAYGo benchmark</t>
-        </is>
-      </c>
-      <c r="R46" s="9" t="inlineStr">
-        <is>
-          <t>UK research and development subsidiary; no employees; functional currency sterling; IFRS as adopted in the UK; not consolidated.</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R46" s="9" t="inlineStr"/>
       <c r="S46" s="9" t="inlineStr"/>
       <c r="T46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>E4-02</t>
+          <t>E3-03</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>M-KOPA UK LIMITED profit for the year</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="n">
-        <v>1040472</v>
+          <t>Duration thresholds: Tier 1 min 4 hours a day and 1 evening hour; Tier 2 min 4 hours and 2 evening hours; affordability attribute met when a standard package of 365 kWh a year costs less than 5% of household income</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>thresholds</t>
+        </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>FY2024 (FY2023: 497,346)</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>M-KOPA UK LIMITED, Annual Report and Accounts, year ended 31 December 2024</t>
+          <t>Beyond Connections: Energy Access Redefined (Technical Report 008/15, conceptualization report)</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>Companies House (company 10229661)</t>
+          <t>ESMAP / World Bank</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>Approved 20 Jun 2025; filed 25 Sep 2025</t>
+          <t>July 2015</t>
         </is>
       </c>
       <c r="I47" s="9" t="inlineStr">
         <is>
-          <t>245b3bf6-companies_house_document.pdf (34 pages, scanned)</t>
+          <t>BEYOND CONNECTIONS  Energy Access Redefined.pdf (244 pages; author's Google Drive, SHA-256 9d23881a...c1d26b)</t>
         </is>
       </c>
       <c r="J47" s="9" t="inlineStr">
         <is>
-          <t>10 (filing page 8)</t>
+          <t>20 (report page 6)</t>
         </is>
       </c>
       <c r="K47" s="9" t="inlineStr">
         <is>
-          <t>Statement of profit or loss</t>
+          <t>Table ES.1</t>
         </is>
       </c>
       <c r="L47" s="9" t="inlineStr">
         <is>
-          <t>Project file (uploaded 3 Oct 2026)</t>
+          <t>Project file (retrieved from the author's Drive, 4 Oct 2026)</t>
         </is>
       </c>
       <c r="M47" s="9" t="inlineStr">
         <is>
-          <t>Audited statutory accounts (auditor KLSA LLP), read page by page</t>
+          <t>Read in the document</t>
         </is>
       </c>
       <c r="N47" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O47" s="9" t="inlineStr">
@@ -4895,42 +4903,44 @@
       </c>
       <c r="P47" s="9" t="inlineStr">
         <is>
+          <t>Ch 2.6</t>
+        </is>
+      </c>
+      <c r="Q47" s="9" t="inlineStr">
+        <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q47" s="9" t="inlineStr">
-        <is>
-          <t>Not used</t>
-        </is>
-      </c>
-      <c r="R47" s="9" t="inlineStr"/>
+      <c r="R47" s="9" t="inlineStr">
+        <is>
+          <t>The MTF affordability test prices a standard consumption package, not a PAYGo instalment; it is a different measure from the payment burden in Ch 2.3.</t>
+        </is>
+      </c>
       <c r="S47" s="9" t="inlineStr"/>
       <c r="T47" s="9" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>E4-03</t>
+          <t>E4-01</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>M-KOPA UK LIMITED parent and ultimate parent: M-Kopa LLC (Delaware); M-Kopa Holdings Limited (London)</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
+          <t>M-KOPA UK LIMITED revenue (sales of carbon credits)</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n">
+        <v>1712776</v>
       </c>
       <c r="D48" s="9" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>FY2024</t>
+          <t>FY2024 (FY2023: 718,100)</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr">
@@ -4955,12 +4965,12 @@
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>3 (filing page 1)</t>
+          <t>10 (filing page 8); 18 (filing page 16, note 2.1)</t>
         </is>
       </c>
       <c r="K48" s="9" t="inlineStr">
         <is>
-          <t>Company information</t>
+          <t>Statement of profit or loss; note 2.1 Sale of carbon credits</t>
         </is>
       </c>
       <c r="L48" s="9" t="inlineStr">
@@ -4985,489 +4995,489 @@
       </c>
       <c r="P48" s="9" t="inlineStr">
         <is>
-          <t>Planned: Ch 15</t>
+          <t>Planned: Ch 15 (as an illustration of entity checking)</t>
         </is>
       </c>
       <c r="Q48" s="9" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Not used: different entity and activity; not a PAYGo benchmark</t>
         </is>
       </c>
       <c r="R48" s="9" t="inlineStr">
         <is>
-          <t>The project's benchmark files attribute the group figures to M-KOPA Holdings Ltd, Companies House 10891868. That number has not been checked against the register.</t>
+          <t>UK research and development subsidiary; no employees; functional currency sterling; IFRS as adopted in the UK; not consolidated.</t>
         </is>
       </c>
       <c r="S48" s="9" t="inlineStr"/>
       <c r="T48" s="9" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>E4-02</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>M-KOPA UK LIMITED profit for the year</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n">
+        <v>1040472</v>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>FY2024 (FY2023: 497,346)</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>M-KOPA UK LIMITED, Annual Report and Accounts, year ended 31 December 2024</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Companies House (company 10229661)</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>Approved 20 Jun 2025; filed 25 Sep 2025</t>
+        </is>
+      </c>
+      <c r="I49" s="9" t="inlineStr">
+        <is>
+          <t>245b3bf6-companies_house_document.pdf (34 pages, scanned)</t>
+        </is>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>10 (filing page 8)</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>Statement of profit or loss</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>Project file (uploaded 3 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>Audited statutory accounts (auditor KLSA LLP), read page by page</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O49" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P49" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q49" s="9" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="R49" s="9" t="inlineStr"/>
+      <c r="S49" s="9" t="inlineStr"/>
+      <c r="T49" s="9" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>E4-03</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>M-KOPA UK LIMITED parent and ultimate parent: M-Kopa LLC (Delaware); M-Kopa Holdings Limited (London)</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>M-KOPA UK LIMITED, Annual Report and Accounts, year ended 31 December 2024</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Companies House (company 10229661)</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>Approved 20 Jun 2025; filed 25 Sep 2025</t>
+        </is>
+      </c>
+      <c r="I50" s="9" t="inlineStr">
+        <is>
+          <t>245b3bf6-companies_house_document.pdf (34 pages, scanned)</t>
+        </is>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>3 (filing page 1)</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>Company information</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>Project file (uploaded 3 Oct 2026)</t>
+        </is>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>Audited statutory accounts (auditor KLSA LLP), read page by page</t>
+        </is>
+      </c>
+      <c r="N50" s="9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O50" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="P50" s="9" t="inlineStr">
+        <is>
+          <t>Planned: Ch 15</t>
+        </is>
+      </c>
+      <c r="Q50" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="R50" s="9" t="inlineStr">
+        <is>
+          <t>The project's benchmark files attribute the group figures to M-KOPA Holdings Ltd, Companies House 10891868. That number has not been checked against the register.</t>
+        </is>
+      </c>
+      <c r="S50" s="9" t="inlineStr"/>
+      <c r="T50" s="9" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>E4-04</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>M-KOPA group revenue FY2024</t>
         </is>
       </c>
-      <c r="C49" s="8" t="n">
+      <c r="C51" s="8" t="n">
         <v>416</v>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D51" s="8" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E51" s="8" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="F49" s="8" t="inlineStr">
+      <c r="F51" s="8" t="inlineStr">
         <is>
           <t>News article citing 'UK filings'</t>
         </is>
       </c>
-      <c r="G49" s="8" t="inlineStr">
+      <c r="G51" s="8" t="inlineStr">
         <is>
           <t>TechCabal</t>
         </is>
       </c>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="H51" s="8" t="inlineStr">
         <is>
           <t>7 Oct 2025</t>
         </is>
       </c>
-      <c r="I49" s="8" t="inlineStr">
+      <c r="I51" s="8" t="inlineStr">
         <is>
           <t>Web article</t>
         </is>
       </c>
-      <c r="J49" s="8" t="inlineStr">
+      <c r="J51" s="8" t="inlineStr">
         <is>
           <t>PAGE TO VERIFY</t>
         </is>
       </c>
-      <c r="K49" s="8" t="inlineStr"/>
-      <c r="L49" s="8" t="inlineStr">
+      <c r="K51" s="8" t="inlineStr"/>
+      <c r="L51" s="8" t="inlineStr">
         <is>
           <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
         </is>
       </c>
-      <c r="M49" s="8" t="inlineStr">
+      <c r="M51" s="8" t="inlineStr">
         <is>
           <t>Secondary report; entity and revenue line not identified</t>
         </is>
       </c>
-      <c r="N49" s="8" t="inlineStr">
+      <c r="N51" s="8" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="O49" s="8" t="inlineStr">
+      <c r="O51" s="8" t="inlineStr">
         <is>
           <t>CONFLICTING SOURCES</t>
         </is>
       </c>
-      <c r="P49" s="8" t="inlineStr">
+      <c r="P51" s="8" t="inlineStr">
         <is>
           <t>Ch 15 (presented as conflicting)</t>
         </is>
       </c>
-      <c r="Q49" s="8" t="inlineStr">
+      <c r="Q51" s="8" t="inlineStr">
         <is>
           <t>Market_Benchmark and Calibration: suspended</t>
         </is>
       </c>
-      <c r="R49" s="8" t="inlineStr">
+      <c r="R51" s="8" t="inlineStr">
         <is>
           <t>Conflicts with E4-05 (USD 253.5m). Not supported by E4-01 (different entity). Resolvable only with the consolidated accounts of the reporting group entity.</t>
         </is>
       </c>
-      <c r="S49" s="8" t="inlineStr">
+      <c r="S51" s="8" t="inlineStr">
         <is>
           <t>M-KOPA|Revenue</t>
         </is>
       </c>
-      <c r="T49" s="8" t="inlineStr">
+      <c r="T51" s="8" t="inlineStr">
         <is>
           <t>SR01</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>E4-05</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>M-KOPA group revenue FY2024</t>
         </is>
       </c>
-      <c r="C50" s="8" t="n">
+      <c r="C52" s="8" t="n">
         <v>253.5</v>
       </c>
-      <c r="D50" s="8" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
         <is>
           <t>FY2024</t>
         </is>
       </c>
-      <c r="F50" s="8" t="inlineStr">
+      <c r="F52" s="8" t="inlineStr">
         <is>
           <t>News article</t>
         </is>
       </c>
-      <c r="G50" s="8" t="inlineStr">
+      <c r="G52" s="8" t="inlineStr">
         <is>
           <t>Kenyan Wall Street</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="I50" s="8" t="inlineStr">
+      <c r="I52" s="8" t="inlineStr">
         <is>
           <t>Web article</t>
         </is>
       </c>
-      <c r="J50" s="8" t="inlineStr">
+      <c r="J52" s="8" t="inlineStr">
         <is>
           <t>PAGE TO VERIFY</t>
         </is>
       </c>
-      <c r="K50" s="8" t="inlineStr"/>
-      <c r="L50" s="8" t="inlineStr">
+      <c r="K52" s="8" t="inlineStr"/>
+      <c r="L52" s="8" t="inlineStr">
         <is>
           <t>https://kenyanwallstreet.com/m-kopa-posts-first-ever-profit-bets-on-e-mobility-for-next-growth-phase/</t>
         </is>
       </c>
-      <c r="M50" s="8" t="inlineStr">
+      <c r="M52" s="8" t="inlineStr">
         <is>
           <t>Secondary report; may be a different revenue line</t>
         </is>
       </c>
-      <c r="N50" s="8" t="inlineStr">
+      <c r="N52" s="8" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="O50" s="8" t="inlineStr">
+      <c r="O52" s="8" t="inlineStr">
         <is>
           <t>CONFLICTING SOURCES</t>
         </is>
       </c>
-      <c r="P50" s="8" t="inlineStr">
+      <c r="P52" s="8" t="inlineStr">
         <is>
           <t>Ch 15 (presented as conflicting)</t>
         </is>
       </c>
-      <c r="Q50" s="8" t="inlineStr">
+      <c r="Q52" s="8" t="inlineStr">
         <is>
           <t>Not used</t>
         </is>
       </c>
-      <c r="R50" s="8" t="inlineStr"/>
-      <c r="S50" s="8" t="inlineStr"/>
-      <c r="T50" s="8" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="R52" s="8" t="inlineStr"/>
+      <c r="S52" s="8" t="inlineStr"/>
+      <c r="T52" s="8" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t>E4-06</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>M-KOPA group revenue growth</t>
         </is>
       </c>
-      <c r="C51" s="7" t="n">
+      <c r="C53" s="7" t="n">
         <v>0.66</v>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>FY2024 vs FY2023</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>News articles</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>TechCabal; Kenyan Wall Street</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>Web articles</t>
         </is>
       </c>
-      <c r="J51" s="7" t="inlineStr">
+      <c r="J53" s="7" t="inlineStr">
         <is>
           <t>PAGE TO VERIFY</t>
         </is>
       </c>
-      <c r="K51" s="7" t="inlineStr"/>
-      <c r="L51" s="7" t="inlineStr">
+      <c r="K53" s="7" t="inlineStr"/>
+      <c r="L53" s="7" t="inlineStr">
         <is>
           <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
         </is>
       </c>
-      <c r="M51" s="7" t="inlineStr">
+      <c r="M53" s="7" t="inlineStr">
         <is>
           <t>Secondary report</t>
         </is>
       </c>
-      <c r="N51" s="7" t="inlineStr">
+      <c r="N53" s="7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="O51" s="7" t="inlineStr">
+      <c r="O53" s="7" t="inlineStr">
         <is>
           <t>PENDING PRIMARY DOCUMENT</t>
         </is>
       </c>
-      <c r="P51" s="7" t="inlineStr">
+      <c r="P53" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q51" s="7" t="inlineStr">
+      <c r="Q53" s="7" t="inlineStr">
         <is>
           <t>Calibration growth reference: suspended</t>
         </is>
       </c>
-      <c r="R51" s="7" t="inlineStr"/>
-      <c r="S51" s="7" t="inlineStr">
+      <c r="R53" s="7" t="inlineStr"/>
+      <c r="S53" s="7" t="inlineStr">
         <is>
           <t>M-KOPA|Revenue growth</t>
         </is>
       </c>
-      <c r="T51" s="7" t="inlineStr">
+      <c r="T53" s="7" t="inlineStr">
         <is>
           <t>SR02</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>E4-07</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>M-KOPA group net profit</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="D52" s="7" t="inlineStr">
-        <is>
-          <t>USD m</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>News article</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>TechCabal</t>
-        </is>
-      </c>
-      <c r="H52" s="7" t="inlineStr">
-        <is>
-          <t>7 Oct 2025</t>
-        </is>
-      </c>
-      <c r="I52" s="7" t="inlineStr">
-        <is>
-          <t>Web article</t>
-        </is>
-      </c>
-      <c r="J52" s="7" t="inlineStr">
-        <is>
-          <t>PAGE TO VERIFY</t>
-        </is>
-      </c>
-      <c r="K52" s="7" t="inlineStr"/>
-      <c r="L52" s="7" t="inlineStr">
-        <is>
-          <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
-        </is>
-      </c>
-      <c r="M52" s="7" t="inlineStr">
-        <is>
-          <t>Secondary report</t>
-        </is>
-      </c>
-      <c r="N52" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="O52" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
-        </is>
-      </c>
-      <c r="P52" s="7" t="inlineStr">
-        <is>
-          <t>Ch 15</t>
-        </is>
-      </c>
-      <c r="Q52" s="7" t="inlineStr">
-        <is>
-          <t>Calibration net margin reference: suspended</t>
-        </is>
-      </c>
-      <c r="R52" s="7" t="inlineStr"/>
-      <c r="S52" s="7" t="inlineStr">
-        <is>
-          <t>M-KOPA|Net profit</t>
-        </is>
-      </c>
-      <c r="T52" s="7" t="inlineStr">
-        <is>
-          <t>SR03</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>E4-08</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>M-KOPA group net result, prior year</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>-24.7 (or -20.6)</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>USD m</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>News articles</t>
-        </is>
-      </c>
-      <c r="G53" s="8" t="inlineStr">
-        <is>
-          <t>TechCabal; Kenyan Wall Street</t>
-        </is>
-      </c>
-      <c r="H53" s="8" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="I53" s="8" t="inlineStr">
-        <is>
-          <t>Web articles</t>
-        </is>
-      </c>
-      <c r="J53" s="8" t="inlineStr">
-        <is>
-          <t>PAGE TO VERIFY</t>
-        </is>
-      </c>
-      <c r="K53" s="8" t="inlineStr"/>
-      <c r="L53" s="8" t="inlineStr">
-        <is>
-          <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
-        </is>
-      </c>
-      <c r="M53" s="8" t="inlineStr">
-        <is>
-          <t>Secondary reports that conflict</t>
-        </is>
-      </c>
-      <c r="N53" s="8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="O53" s="8" t="inlineStr">
-        <is>
-          <t>CONFLICTING SOURCES</t>
-        </is>
-      </c>
-      <c r="P53" s="8" t="inlineStr">
-        <is>
-          <t>Ch 15</t>
-        </is>
-      </c>
-      <c r="Q53" s="8" t="inlineStr">
-        <is>
-          <t>Not used</t>
-        </is>
-      </c>
-      <c r="R53" s="8" t="inlineStr"/>
-      <c r="S53" s="8" t="inlineStr"/>
-      <c r="T53" s="8" t="inlineStr">
-        <is>
-          <t>SR04</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>E5-01</t>
+          <t>E4-07</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Sun King cumulative solar loans</t>
+          <t>M-KOPA group net profit</t>
         </is>
       </c>
       <c r="C54" s="7" t="n">
-        <v>1300</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
@@ -5476,27 +5486,27 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Cumulative to Jul 2025</t>
+          <t>FY2024</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Citi press release on the Sun King securitisation</t>
+          <t>News article</t>
         </is>
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>TechCabal</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>7 Oct 2025</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>Press release (not read in this project)</t>
+          <t>Web article</t>
         </is>
       </c>
       <c r="J54" s="7" t="inlineStr">
@@ -5507,17 +5517,17 @@
       <c r="K54" s="7" t="inlineStr"/>
       <c r="L54" s="7" t="inlineStr">
         <is>
-          <t>https://www.citigroup.com/global/news/press-release/2025/citi-sun-king-securitization-deliver-solar-million-kenyans</t>
+          <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
         </is>
       </c>
       <c r="M54" s="7" t="inlineStr">
         <is>
-          <t>Company disclosure recorded from earlier research</t>
+          <t>Secondary report</t>
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="O54" s="7" t="inlineStr">
@@ -5527,131 +5537,129 @@
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
-          <t>Ch 12, 15</t>
+          <t>Ch 15</t>
         </is>
       </c>
       <c r="Q54" s="7" t="inlineStr">
         <is>
-          <t>Market_Benchmark (shown, flagged)</t>
+          <t>Calibration net margin reference: suspended</t>
         </is>
       </c>
       <c r="R54" s="7" t="inlineStr"/>
       <c r="S54" s="7" t="inlineStr">
         <is>
-          <t>Sun King|Cumulative solar loans</t>
+          <t>M-KOPA|Net profit</t>
         </is>
       </c>
       <c r="T54" s="7" t="inlineStr">
         <is>
-          <t>SR05</t>
+          <t>SR03</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>E5-02</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>Sun King cumulative loan customers (cumulative, not active)</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>million</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="inlineStr">
-        <is>
-          <t>Cumulative to Jul 2025</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Citi press release</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>Citigroup</t>
-        </is>
-      </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>E4-08</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>M-KOPA group net result, prior year</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>-24.7 (or -20.6)</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>News articles</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>TechCabal; Kenyan Wall Street</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>Press release (not read)</t>
-        </is>
-      </c>
-      <c r="J55" s="7" t="inlineStr">
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>Web articles</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="inlineStr">
         <is>
           <t>PAGE TO VERIFY</t>
         </is>
       </c>
-      <c r="K55" s="7" t="inlineStr"/>
-      <c r="L55" s="7" t="inlineStr">
-        <is>
-          <t>https://www.citigroup.com/global/news/press-release/2025/citi-sun-king-securitization-deliver-solar-million-kenyans</t>
-        </is>
-      </c>
-      <c r="M55" s="7" t="inlineStr">
-        <is>
-          <t>Company disclosure recorded from earlier research</t>
-        </is>
-      </c>
-      <c r="N55" s="7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="O55" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
-        </is>
-      </c>
-      <c r="P55" s="7" t="inlineStr">
-        <is>
-          <t>Ch 12, 15</t>
-        </is>
-      </c>
-      <c r="Q55" s="7" t="inlineStr">
-        <is>
-          <t>Market_Benchmark (shown, flagged)</t>
-        </is>
-      </c>
-      <c r="R55" s="7" t="inlineStr"/>
-      <c r="S55" s="7" t="inlineStr">
-        <is>
-          <t>Sun King|Cumulative loan customers</t>
-        </is>
-      </c>
-      <c r="T55" s="7" t="inlineStr">
-        <is>
-          <t>SR06</t>
+      <c r="K55" s="8" t="inlineStr"/>
+      <c r="L55" s="8" t="inlineStr">
+        <is>
+          <t>https://techcabal.com/2025/10/07/m-kopa-turns-first-ever-profit-revenue-surges-66-416/</t>
+        </is>
+      </c>
+      <c r="M55" s="8" t="inlineStr">
+        <is>
+          <t>Secondary reports that conflict</t>
+        </is>
+      </c>
+      <c r="N55" s="8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O55" s="8" t="inlineStr">
+        <is>
+          <t>CONFLICTING SOURCES</t>
+        </is>
+      </c>
+      <c r="P55" s="8" t="inlineStr">
+        <is>
+          <t>Ch 15</t>
+        </is>
+      </c>
+      <c r="Q55" s="8" t="inlineStr">
+        <is>
+          <t>Not used</t>
+        </is>
+      </c>
+      <c r="R55" s="8" t="inlineStr"/>
+      <c r="S55" s="8" t="inlineStr"/>
+      <c r="T55" s="8" t="inlineStr">
+        <is>
+          <t>SR04</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>E5-03</t>
+          <t>E5-01</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>Sun King local-currency securitisation in Kenya</t>
+          <t>Sun King cumulative solar loans</t>
         </is>
       </c>
       <c r="C56" s="7" t="n">
-        <v>130</v>
+        <v>1300</v>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
@@ -5660,27 +5668,27 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>May 2023</t>
+          <t>Cumulative to Jul 2025</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Sun King news release</t>
+          <t>Citi press release on the Sun King securitisation</t>
         </is>
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Sun King</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="I56" s="7" t="inlineStr">
         <is>
-          <t>News release (not read)</t>
+          <t>Press release (not read in this project)</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
@@ -5691,7 +5699,7 @@
       <c r="K56" s="7" t="inlineStr"/>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>https://sunking.com/news-blog/sun-king-and-citi-close-first-130-million-securitisation-to-broaden-access-to-finance-for-off-grid-solar-in-kenya/</t>
+          <t>https://www.citigroup.com/global/news/press-release/2025/citi-sun-king-securitization-deliver-solar-million-kenyans</t>
         </is>
       </c>
       <c r="M56" s="7" t="inlineStr">
@@ -5711,64 +5719,68 @@
       </c>
       <c r="P56" s="7" t="inlineStr">
         <is>
-          <t>Ch 3.11, 11, 12</t>
+          <t>Ch 12, 15</t>
         </is>
       </c>
       <c r="Q56" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Market_Benchmark (shown, flagged)</t>
         </is>
       </c>
       <c r="R56" s="7" t="inlineStr"/>
-      <c r="S56" s="7" t="inlineStr"/>
+      <c r="S56" s="7" t="inlineStr">
+        <is>
+          <t>Sun King|Cumulative solar loans</t>
+        </is>
+      </c>
       <c r="T56" s="7" t="inlineStr">
         <is>
-          <t>SR07</t>
+          <t>SR05</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>E5-04</t>
+          <t>E5-02</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Sun King local-currency securitisation in Kenya (KES 20.1bn)</t>
+          <t>Sun King cumulative loan customers (cumulative, not active)</t>
         </is>
       </c>
       <c r="C57" s="7" t="n">
-        <v>156</v>
+        <v>10</v>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>USD m</t>
+          <t>million</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Jul 2025</t>
+          <t>Cumulative to Jul 2025</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Citi release; trade press</t>
+          <t>Citi press release</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Citigroup; pv magazine</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>29 Jul 2025</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>Release and article (not read)</t>
+          <t>Press release (not read)</t>
         </is>
       </c>
       <c r="J57" s="7" t="inlineStr">
@@ -5779,12 +5791,12 @@
       <c r="K57" s="7" t="inlineStr"/>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>https://www.pv-magazine.com/2025/07/29/sun-king-closes-156m-off-grid-solar-deal-in-kenya/</t>
+          <t>https://www.citigroup.com/global/news/press-release/2025/citi-sun-king-securitization-deliver-solar-million-kenyans</t>
         </is>
       </c>
       <c r="M57" s="7" t="inlineStr">
         <is>
-          <t>Company disclosure and secondary report recorded from earlier research</t>
+          <t>Company disclosure recorded from earlier research</t>
         </is>
       </c>
       <c r="N57" s="7" t="inlineStr">
@@ -5799,7 +5811,7 @@
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
-          <t>Ch 3.11, 11, 12</t>
+          <t>Ch 12, 15</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
@@ -5810,96 +5822,116 @@
       <c r="R57" s="7" t="inlineStr"/>
       <c r="S57" s="7" t="inlineStr">
         <is>
-          <t>Sun King|Securitisation 2025</t>
+          <t>Sun King|Cumulative loan customers</t>
         </is>
       </c>
       <c r="T57" s="7" t="inlineStr">
         <is>
-          <t>SR08</t>
+          <t>SR06</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="11" t="inlineStr">
-        <is>
-          <t>E5-05</t>
-        </is>
-      </c>
-      <c r="B58" s="11" t="inlineStr">
-        <is>
-          <t>Sun King MSME bond</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>E5-03</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Sun King local-currency securitisation in Kenya</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="F58" s="11" t="inlineStr">
-        <is>
-          <t>None found</t>
-        </is>
-      </c>
-      <c r="G58" s="11" t="inlineStr"/>
-      <c r="H58" s="11" t="inlineStr"/>
-      <c r="I58" s="11" t="inlineStr"/>
-      <c r="J58" s="11" t="inlineStr"/>
-      <c r="K58" s="11" t="inlineStr"/>
-      <c r="L58" s="11" t="inlineStr"/>
-      <c r="M58" s="11" t="inlineStr">
-        <is>
-          <t>No public source found</t>
-        </is>
-      </c>
-      <c r="N58" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O58" s="11" t="inlineStr">
-        <is>
-          <t>NOT USED</t>
-        </is>
-      </c>
-      <c r="P58" s="11" t="inlineStr">
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>May 2023</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Sun King news release</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Sun King</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>News release (not read)</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>PAGE TO VERIFY</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr"/>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>https://sunking.com/news-blog/sun-king-and-citi-close-first-130-million-securitisation-to-broaden-access-to-finance-for-off-grid-solar-in-kenya/</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>Company disclosure recorded from earlier research</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O58" s="7" t="inlineStr">
+        <is>
+          <t>PENDING PRIMARY DOCUMENT</t>
+        </is>
+      </c>
+      <c r="P58" s="7" t="inlineStr">
+        <is>
+          <t>Ch 3.11, 11, 12</t>
+        </is>
+      </c>
+      <c r="Q58" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q58" s="11" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="R58" s="11" t="inlineStr"/>
-      <c r="S58" s="11" t="inlineStr"/>
-      <c r="T58" s="11" t="inlineStr">
-        <is>
-          <t>SR09</t>
+      <c r="R58" s="7" t="inlineStr"/>
+      <c r="S58" s="7" t="inlineStr"/>
+      <c r="T58" s="7" t="inlineStr">
+        <is>
+          <t>SR07</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>E6-01</t>
+          <t>E5-04</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>d.light securitisation purchasing capacity since 2020 (five facilities; purchasing capacity, not debt raised)</t>
+          <t>Sun King local-currency securitisation in Kenya (KES 20.1bn)</t>
         </is>
       </c>
       <c r="C59" s="7" t="n">
-        <v>718</v>
+        <v>156</v>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
@@ -5908,27 +5940,27 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>2020 to Jul 2024</t>
+          <t>Jul 2025</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>News article</t>
+          <t>Citi release; trade press</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Techpoint Africa</t>
+          <t>Citigroup; pv magazine</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>17 Jul 2024</t>
+          <t>29 Jul 2025</t>
         </is>
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>Web article</t>
+          <t>Release and article (not read)</t>
         </is>
       </c>
       <c r="J59" s="7" t="inlineStr">
@@ -5939,17 +5971,17 @@
       <c r="K59" s="7" t="inlineStr"/>
       <c r="L59" s="7" t="inlineStr">
         <is>
-          <t>https://techpoint.africa/2024/07/17/d-light-raises-176m/</t>
+          <t>https://www.pv-magazine.com/2025/07/29/sun-king-closes-156m-off-grid-solar-deal-in-kenya/</t>
         </is>
       </c>
       <c r="M59" s="7" t="inlineStr">
         <is>
-          <t>Secondary report</t>
+          <t>Company disclosure and secondary report recorded from earlier research</t>
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O59" s="7" t="inlineStr">
@@ -5959,7 +5991,7 @@
       </c>
       <c r="P59" s="7" t="inlineStr">
         <is>
-          <t>Ch 3.11, 11, 12, 15</t>
+          <t>Ch 3.11, 11, 12</t>
         </is>
       </c>
       <c r="Q59" s="7" t="inlineStr">
@@ -5970,149 +6002,125 @@
       <c r="R59" s="7" t="inlineStr"/>
       <c r="S59" s="7" t="inlineStr">
         <is>
-          <t>d.light|Securitisation purchasing capacity since 2020</t>
+          <t>Sun King|Securitisation 2025</t>
         </is>
       </c>
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>SR10</t>
+          <t>SR08</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>E6-02</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>d.light multi-currency securitisation facility</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="n">
-        <v>176</v>
-      </c>
-      <c r="D60" s="7" t="inlineStr">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>E5-05</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>Sun King MSME bond</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="E60" s="7" t="inlineStr">
-        <is>
-          <t>Jul 2024</t>
-        </is>
-      </c>
-      <c r="F60" s="7" t="inlineStr">
-        <is>
-          <t>News articles</t>
-        </is>
-      </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>Techpoint Africa; WeeTracker</t>
-        </is>
-      </c>
-      <c r="H60" s="7" t="inlineStr">
-        <is>
-          <t>17 Jul 2024</t>
-        </is>
-      </c>
-      <c r="I60" s="7" t="inlineStr">
-        <is>
-          <t>Web articles</t>
-        </is>
-      </c>
-      <c r="J60" s="7" t="inlineStr">
-        <is>
-          <t>PAGE TO VERIFY</t>
-        </is>
-      </c>
-      <c r="K60" s="7" t="inlineStr"/>
-      <c r="L60" s="7" t="inlineStr">
-        <is>
-          <t>https://techpoint.africa/2024/07/17/d-light-raises-176m/</t>
-        </is>
-      </c>
-      <c r="M60" s="7" t="inlineStr">
-        <is>
-          <t>Secondary report</t>
-        </is>
-      </c>
-      <c r="N60" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="O60" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
-        </is>
-      </c>
-      <c r="P60" s="7" t="inlineStr">
-        <is>
-          <t>Ch 12</t>
-        </is>
-      </c>
-      <c r="Q60" s="7" t="inlineStr">
-        <is>
-          <t>Market_Benchmark (shown, flagged)</t>
-        </is>
-      </c>
-      <c r="R60" s="7" t="inlineStr"/>
-      <c r="S60" s="7" t="inlineStr">
-        <is>
-          <t>d.light|Securitisation facility 2024</t>
-        </is>
-      </c>
-      <c r="T60" s="7" t="inlineStr">
-        <is>
-          <t>SR11</t>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr"/>
+      <c r="H60" s="11" t="inlineStr"/>
+      <c r="I60" s="11" t="inlineStr"/>
+      <c r="J60" s="11" t="inlineStr"/>
+      <c r="K60" s="11" t="inlineStr"/>
+      <c r="L60" s="11" t="inlineStr"/>
+      <c r="M60" s="11" t="inlineStr">
+        <is>
+          <t>No public source found</t>
+        </is>
+      </c>
+      <c r="N60" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="O60" s="11" t="inlineStr">
+        <is>
+          <t>NOT USED</t>
+        </is>
+      </c>
+      <c r="P60" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q60" s="11" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="R60" s="11" t="inlineStr"/>
+      <c r="S60" s="11" t="inlineStr"/>
+      <c r="T60" s="11" t="inlineStr">
+        <is>
+          <t>SR09</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>E6-03</t>
+          <t>E6-01</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>d.light revenue growth</t>
+          <t>d.light securitisation purchasing capacity since 2020 (five facilities; purchasing capacity, not debt raised)</t>
         </is>
       </c>
       <c r="C61" s="7" t="n">
-        <v>0.41</v>
+        <v>718</v>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>USD m</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>H1 2023 vs H1 2022</t>
+          <t>2020 to Jul 2024</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>d.light press release</t>
+          <t>News article</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>d.light via PR Newswire</t>
+          <t>Techpoint Africa</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>Sep 2023</t>
+          <t>17 Jul 2024</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>Press release (not read)</t>
+          <t>Web article</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
@@ -6123,17 +6131,17 @@
       <c r="K61" s="7" t="inlineStr"/>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.co.uk/news-releases/dlight-revenues-surge-by-41-percent-in-first-six-months-of-2023-driven-by-143-percent-growth-in-nigeria-301919233.html</t>
+          <t>https://techpoint.africa/2024/07/17/d-light-raises-176m/</t>
         </is>
       </c>
       <c r="M61" s="7" t="inlineStr">
         <is>
-          <t>Company disclosure recorded from earlier research</t>
+          <t>Secondary report</t>
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="O61" s="7" t="inlineStr">
@@ -6143,7 +6151,7 @@
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Ch 3.11, 11, 12, 15</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
@@ -6154,164 +6162,170 @@
       <c r="R61" s="7" t="inlineStr"/>
       <c r="S61" s="7" t="inlineStr">
         <is>
-          <t>d.light|Revenue growth</t>
+          <t>d.light|Securitisation purchasing capacity since 2020</t>
         </is>
       </c>
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>SR12</t>
+          <t>SR10</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="11" t="inlineStr">
-        <is>
-          <t>E6-04</t>
-        </is>
-      </c>
-      <c r="B62" s="11" t="inlineStr">
-        <is>
-          <t>d.light revenue (third-party estimate)</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="n">
-        <v>301.2</v>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>E6-02</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>d.light multi-currency securitisation facility</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>176</v>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>USD m</t>
         </is>
       </c>
-      <c r="E62" s="11" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="F62" s="11" t="inlineStr">
-        <is>
-          <t>Company database</t>
-        </is>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>bitscale.ai</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Web page</t>
-        </is>
-      </c>
-      <c r="J62" s="11" t="inlineStr"/>
-      <c r="K62" s="11" t="inlineStr"/>
-      <c r="L62" s="11" t="inlineStr">
-        <is>
-          <t>https://www.bitscale.ai/directory/dlight</t>
-        </is>
-      </c>
-      <c r="M62" s="11" t="inlineStr">
-        <is>
-          <t>Third-party estimate, method not stated</t>
-        </is>
-      </c>
-      <c r="N62" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O62" s="11" t="inlineStr">
-        <is>
-          <t>NOT USED</t>
-        </is>
-      </c>
-      <c r="P62" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Q62" s="11" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="R62" s="11" t="inlineStr"/>
-      <c r="S62" s="11" t="inlineStr"/>
-      <c r="T62" s="11" t="inlineStr">
-        <is>
-          <t>SR13</t>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Jul 2024</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>News articles</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Techpoint Africa; WeeTracker</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>17 Jul 2024</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>Web articles</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>PAGE TO VERIFY</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr"/>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>https://techpoint.africa/2024/07/17/d-light-raises-176m/</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>Secondary report</t>
+        </is>
+      </c>
+      <c r="N62" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O62" s="7" t="inlineStr">
+        <is>
+          <t>PENDING PRIMARY DOCUMENT</t>
+        </is>
+      </c>
+      <c r="P62" s="7" t="inlineStr">
+        <is>
+          <t>Ch 12</t>
+        </is>
+      </c>
+      <c r="Q62" s="7" t="inlineStr">
+        <is>
+          <t>Market_Benchmark (shown, flagged)</t>
+        </is>
+      </c>
+      <c r="R62" s="7" t="inlineStr"/>
+      <c r="S62" s="7" t="inlineStr">
+        <is>
+          <t>d.light|Securitisation facility 2024</t>
+        </is>
+      </c>
+      <c r="T62" s="7" t="inlineStr">
+        <is>
+          <t>SR11</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>E7-01</t>
+          <t>E6-03</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>BBOXX LTD (07177839): appointment of administrators</t>
-        </is>
-      </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>19 May 2025</t>
-        </is>
+          <t>d.light revenue growth</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>0.41</v>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>%</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>H1 2023 vs H1 2022</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Notice of appointment of administrators</t>
+          <t>d.light press release</t>
         </is>
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>The Gazette</t>
+          <t>d.light via PR Newswire</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>2025 (to verify)</t>
+          <t>Sep 2023</t>
         </is>
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>Gazette notice 4891954 (not held)</t>
+          <t>Press release (not read)</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>PAGE TO VERIFY</t>
         </is>
       </c>
       <c r="K63" s="7" t="inlineStr"/>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>https://www.thegazette.co.uk/notice/4891954 (not opened from this environment)</t>
+          <t>https://www.prnewswire.co.uk/news-releases/dlight-revenues-surge-by-41-percent-in-first-six-months-of-2023-driven-by-143-percent-growth-in-nigeria-301919233.html</t>
         </is>
       </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
-          <t>Date recorded from earlier research (Gazette and administrator's announcement); notice not read in this project</t>
+          <t>Company disclosure recorded from earlier research</t>
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="O63" s="7" t="inlineStr">
@@ -6321,144 +6335,144 @@
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
-          <t>Ch 1.6, 14</t>
+          <t>None</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>Company_Cases text</t>
-        </is>
-      </c>
-      <c r="R63" s="7" t="inlineStr">
-        <is>
-          <t>The date must be the date of appointment stated in the formal notice, not a petition, hearing, publication or creditors' meeting date.</t>
-        </is>
-      </c>
-      <c r="S63" s="7" t="inlineStr"/>
+          <t>Market_Benchmark (shown, flagged)</t>
+        </is>
+      </c>
+      <c r="R63" s="7" t="inlineStr"/>
+      <c r="S63" s="7" t="inlineStr">
+        <is>
+          <t>d.light|Revenue growth</t>
+        </is>
+      </c>
       <c r="T63" s="7" t="inlineStr">
         <is>
-          <t>SR15</t>
+          <t>SR12</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>E7-02</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>BBOXX LTD (07177839): latest filed accounts made up to 31 Dec 2022; FY2023 accounts overdue; status in administration</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D64" s="7" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>Companies House register</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
-        <is>
-          <t>Companies House</t>
-        </is>
-      </c>
-      <c r="H64" s="7" t="inlineStr">
-        <is>
-          <t>2025 (to verify)</t>
-        </is>
-      </c>
-      <c r="I64" s="7" t="inlineStr">
-        <is>
-          <t>Register entry (not opened)</t>
-        </is>
-      </c>
-      <c r="J64" s="7" t="inlineStr"/>
-      <c r="K64" s="7" t="inlineStr"/>
-      <c r="L64" s="7" t="inlineStr">
-        <is>
-          <t>https://find-and-update.company-information.service.gov.uk/company/07177839 (not opened from this environment)</t>
-        </is>
-      </c>
-      <c r="M64" s="7" t="inlineStr">
-        <is>
-          <t>Recorded from earlier research</t>
-        </is>
-      </c>
-      <c r="N64" s="7" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="O64" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
-        </is>
-      </c>
-      <c r="P64" s="7" t="inlineStr">
-        <is>
-          <t>Ch 1.6</t>
-        </is>
-      </c>
-      <c r="Q64" s="7" t="inlineStr">
-        <is>
-          <t>Company_Cases text</t>
-        </is>
-      </c>
-      <c r="R64" s="7" t="inlineStr"/>
-      <c r="S64" s="7" t="inlineStr"/>
-      <c r="T64" s="7" t="inlineStr">
-        <is>
-          <t>SR14</t>
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>E6-04</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>d.light revenue (third-party estimate)</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="n">
+        <v>301.2</v>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>Company database</t>
+        </is>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>bitscale.ai</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>Web page</t>
+        </is>
+      </c>
+      <c r="J64" s="11" t="inlineStr"/>
+      <c r="K64" s="11" t="inlineStr"/>
+      <c r="L64" s="11" t="inlineStr">
+        <is>
+          <t>https://www.bitscale.ai/directory/dlight</t>
+        </is>
+      </c>
+      <c r="M64" s="11" t="inlineStr">
+        <is>
+          <t>Third-party estimate, method not stated</t>
+        </is>
+      </c>
+      <c r="N64" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="O64" s="11" t="inlineStr">
+        <is>
+          <t>NOT USED</t>
+        </is>
+      </c>
+      <c r="P64" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q64" s="11" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="R64" s="11" t="inlineStr"/>
+      <c r="S64" s="11" t="inlineStr"/>
+      <c r="T64" s="11" t="inlineStr">
+        <is>
+          <t>SR13</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>E8-01</t>
+          <t>E7-01</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Off-grid solar investment in 2024, down about 30%</t>
-        </is>
-      </c>
-      <c r="C65" s="7" t="n">
-        <v>299</v>
+          <t>BBOXX LTD (07177839): appointment of administrators</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>19 May 2025</t>
+        </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>USD m</t>
+          <t>date</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>GOGLA investment data (as reported)</t>
+          <t>Notice of appointment of administrators</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>GOGLA</t>
+          <t>The Gazette</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -6468,24 +6482,28 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>Not held</t>
+          <t>Gazette notice 4891954 (not held)</t>
         </is>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>PAGE TO VERIFY</t>
+          <t>Notice</t>
         </is>
       </c>
       <c r="K65" s="7" t="inlineStr"/>
-      <c r="L65" s="7" t="inlineStr"/>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>https://www.thegazette.co.uk/notice/4891954 (not opened from this environment)</t>
+        </is>
+      </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
-          <t>Secondary report</t>
+          <t>Date recorded from earlier research (Gazette and administrator's announcement); notice not read in this project</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="O65" s="7" t="inlineStr">
@@ -6495,85 +6513,87 @@
       </c>
       <c r="P65" s="7" t="inlineStr">
         <is>
-          <t>Ch 11.1, 14</t>
+          <t>Ch 1.6, 14</t>
         </is>
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Company_Cases text</t>
         </is>
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>Consistency only, not verification: E1-17 gives USD 425m for 2023, and 425 x 0.7 is about 298.</t>
+          <t>The date must be the date of appointment stated in the formal notice, not a petition, hearing, publication or creditors' meeting date.</t>
         </is>
       </c>
       <c r="S65" s="7" t="inlineStr"/>
-      <c r="T65" s="7" t="inlineStr"/>
+      <c r="T65" s="7" t="inlineStr">
+        <is>
+          <t>SR15</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>E9-01</t>
+          <t>E7-02</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>ZOLA Electric financing round (USD 45m equity, USD 45m debt)</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="n">
-        <v>90</v>
+          <t>BBOXX LTD (07177839): latest filed accounts made up to 31 Dec 2022; FY2023 accounts overdue; status in administration</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>USD m</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Sep 2021</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>News article</t>
+          <t>Companies House register</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>Companies House</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>23 Sep 2021</t>
+          <t>2025 (to verify)</t>
         </is>
       </c>
       <c r="I66" s="7" t="inlineStr">
         <is>
-          <t>Web article</t>
-        </is>
-      </c>
-      <c r="J66" s="7" t="inlineStr">
-        <is>
-          <t>PAGE TO VERIFY</t>
-        </is>
-      </c>
+          <t>Register entry (not opened)</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr"/>
       <c r="K66" s="7" t="inlineStr"/>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2021/09/23/zola-electric-closes-90m-funding-round-to-scale-technology-and-enter-new-markets</t>
+          <t>https://find-and-update.company-information.service.gov.uk/company/07177839 (not opened from this environment)</t>
         </is>
       </c>
       <c r="M66" s="7" t="inlineStr">
         <is>
-          <t>Secondary report</t>
+          <t>Recorded from earlier research</t>
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="O66" s="7" t="inlineStr">
@@ -6583,65 +6603,59 @@
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Ch 1.6</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>Market_Benchmark (shown, flagged)</t>
+          <t>Company_Cases text</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr"/>
-      <c r="S66" s="7" t="inlineStr">
-        <is>
-          <t>ZOLA Electric|Financing round</t>
-        </is>
-      </c>
+      <c r="S66" s="7" t="inlineStr"/>
       <c r="T66" s="7" t="inlineStr">
         <is>
-          <t>SR18</t>
+          <t>SR14</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>E10-01</t>
+          <t>E8-01</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>SEforALL Universal Energy Facility pays results-based finance per verified connection</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>qualitative</t>
-        </is>
+          <t>Off-grid solar investment in 2024, down about 30%</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>299</v>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>USD m</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>SEforALL (as reported)</t>
+          <t>GOGLA investment data (as reported)</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>SEforALL</t>
+          <t>GOGLA</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>to verify</t>
+          <t>2025 (to verify)</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -6658,7 +6672,7 @@
       <c r="L67" s="7" t="inlineStr"/>
       <c r="M67" s="7" t="inlineStr">
         <is>
-          <t>Secondary description</t>
+          <t>Secondary report</t>
         </is>
       </c>
       <c r="N67" s="7" t="inlineStr">
@@ -6673,7 +6687,7 @@
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>Ch 13.2</t>
+          <t>Ch 11.1, 14</t>
         </is>
       </c>
       <c r="Q67" s="7" t="inlineStr">
@@ -6681,183 +6695,215 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R67" s="7" t="inlineStr"/>
+      <c r="R67" s="7" t="inlineStr">
+        <is>
+          <t>Consistency only, not verification: E1-17 gives USD 425m for 2023, and 425 x 0.7 is about 298.</t>
+        </is>
+      </c>
       <c r="S67" s="7" t="inlineStr"/>
       <c r="T67" s="7" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="11" t="inlineStr">
-        <is>
-          <t>X-01</t>
-        </is>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>Pawame SHS financed</t>
-        </is>
-      </c>
-      <c r="C68" s="11" t="n">
-        <v>18700</v>
-      </c>
-      <c r="D68" s="11" t="inlineStr">
-        <is>
-          <t>units</t>
-        </is>
-      </c>
-      <c r="E68" s="11" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>E9-01</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>ZOLA Electric financing round (USD 45m equity, USD 45m debt)</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>News article</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>23 Sep 2021</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>Web article</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>PAGE TO VERIFY</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr"/>
+      <c r="L68" s="7" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2021/09/23/zola-electric-closes-90m-funding-round-to-scale-technology-and-enter-new-markets</t>
+        </is>
+      </c>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>Secondary report</t>
+        </is>
+      </c>
+      <c r="N68" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="O68" s="7" t="inlineStr">
+        <is>
+          <t>PENDING PRIMARY DOCUMENT</t>
+        </is>
+      </c>
+      <c r="P68" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q68" s="7" t="inlineStr">
+        <is>
+          <t>Market_Benchmark (shown, flagged)</t>
+        </is>
+      </c>
+      <c r="R68" s="7" t="inlineStr"/>
+      <c r="S68" s="7" t="inlineStr">
+        <is>
+          <t>ZOLA Electric|Financing round</t>
+        </is>
+      </c>
+      <c r="T68" s="7" t="inlineStr">
+        <is>
+          <t>SR18</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>E10-01</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>SEforALL Universal Energy Facility pays results-based finance per verified connection</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>None found</t>
-        </is>
-      </c>
-      <c r="G68" s="11" t="inlineStr"/>
-      <c r="H68" s="11" t="inlineStr"/>
-      <c r="I68" s="11" t="inlineStr"/>
-      <c r="J68" s="11" t="inlineStr"/>
-      <c r="K68" s="11" t="inlineStr"/>
-      <c r="L68" s="11" t="inlineStr"/>
-      <c r="M68" s="11" t="inlineStr">
-        <is>
-          <t>No public source found</t>
-        </is>
-      </c>
-      <c r="N68" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O68" s="11" t="inlineStr">
-        <is>
-          <t>NOT USED</t>
-        </is>
-      </c>
-      <c r="P68" s="11" t="inlineStr">
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>SEforALL (as reported)</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>SEforALL</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>to verify</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>Not held</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>PAGE TO VERIFY</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr"/>
+      <c r="L69" s="7" t="inlineStr"/>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>Secondary description</t>
+        </is>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="O69" s="7" t="inlineStr">
+        <is>
+          <t>PENDING PRIMARY DOCUMENT</t>
+        </is>
+      </c>
+      <c r="P69" s="7" t="inlineStr">
+        <is>
+          <t>Ch 13.2</t>
+        </is>
+      </c>
+      <c r="Q69" s="7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q68" s="11" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="R68" s="11" t="inlineStr"/>
-      <c r="S68" s="11" t="inlineStr">
-        <is>
-          <t>Pawame|SHS financed</t>
-        </is>
-      </c>
-      <c r="T68" s="11" t="inlineStr">
-        <is>
-          <t>SR16</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="11" t="inlineStr">
-        <is>
-          <t>X-02</t>
-        </is>
-      </c>
-      <c r="B69" s="11" t="inlineStr">
-        <is>
-          <t>Pawame active customers</t>
-        </is>
-      </c>
-      <c r="C69" s="11" t="n">
-        <v>16000</v>
-      </c>
-      <c r="D69" s="11" t="inlineStr">
-        <is>
-          <t>customers</t>
-        </is>
-      </c>
-      <c r="E69" s="11" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F69" s="11" t="inlineStr">
-        <is>
-          <t>None found</t>
-        </is>
-      </c>
-      <c r="G69" s="11" t="inlineStr"/>
-      <c r="H69" s="11" t="inlineStr"/>
-      <c r="I69" s="11" t="inlineStr"/>
-      <c r="J69" s="11" t="inlineStr"/>
-      <c r="K69" s="11" t="inlineStr"/>
-      <c r="L69" s="11" t="inlineStr"/>
-      <c r="M69" s="11" t="inlineStr">
-        <is>
-          <t>No public source found</t>
-        </is>
-      </c>
-      <c r="N69" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="O69" s="11" t="inlineStr">
-        <is>
-          <t>NOT USED</t>
-        </is>
-      </c>
-      <c r="P69" s="11" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Q69" s="11" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="R69" s="11" t="inlineStr"/>
-      <c r="S69" s="11" t="inlineStr">
-        <is>
-          <t>Pawame|Active customers</t>
-        </is>
-      </c>
-      <c r="T69" s="11" t="inlineStr">
-        <is>
-          <t>SR17</t>
-        </is>
-      </c>
+      <c r="R69" s="7" t="inlineStr"/>
+      <c r="S69" s="7" t="inlineStr"/>
+      <c r="T69" s="7" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>X-01</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
         <is>
-          <t>IFC / AFC material on PAYGo receivables financing</t>
-        </is>
-      </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>reference</t>
-        </is>
+          <t>Pawame SHS financed</t>
+        </is>
+      </c>
+      <c r="C70" s="11" t="n">
+        <v>18700</v>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>units</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>various</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F70" s="11" t="inlineStr">
         <is>
-          <t>Not identified</t>
+          <t>None found</t>
         </is>
       </c>
       <c r="G70" s="11" t="inlineStr"/>
@@ -6868,39 +6914,185 @@
       <c r="L70" s="11" t="inlineStr"/>
       <c r="M70" s="11" t="inlineStr">
         <is>
+          <t>No public source found</t>
+        </is>
+      </c>
+      <c r="N70" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="O70" s="11" t="inlineStr">
+        <is>
+          <t>NOT USED</t>
+        </is>
+      </c>
+      <c r="P70" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q70" s="11" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="R70" s="11" t="inlineStr"/>
+      <c r="S70" s="11" t="inlineStr">
+        <is>
+          <t>Pawame|SHS financed</t>
+        </is>
+      </c>
+      <c r="T70" s="11" t="inlineStr">
+        <is>
+          <t>SR16</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>X-02</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>Pawame active customers</t>
+        </is>
+      </c>
+      <c r="C71" s="11" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
+        <is>
+          <t>customers</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>None found</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="inlineStr"/>
+      <c r="H71" s="11" t="inlineStr"/>
+      <c r="I71" s="11" t="inlineStr"/>
+      <c r="J71" s="11" t="inlineStr"/>
+      <c r="K71" s="11" t="inlineStr"/>
+      <c r="L71" s="11" t="inlineStr"/>
+      <c r="M71" s="11" t="inlineStr">
+        <is>
+          <t>No public source found</t>
+        </is>
+      </c>
+      <c r="N71" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="O71" s="11" t="inlineStr">
+        <is>
+          <t>NOT USED</t>
+        </is>
+      </c>
+      <c r="P71" s="11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Q71" s="11" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="R71" s="11" t="inlineStr"/>
+      <c r="S71" s="11" t="inlineStr">
+        <is>
+          <t>Pawame|Active customers</t>
+        </is>
+      </c>
+      <c r="T71" s="11" t="inlineStr">
+        <is>
+          <t>SR17</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>IFC / AFC material on PAYGo receivables financing</t>
+        </is>
+      </c>
+      <c r="C72" s="11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>various</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>Not identified</t>
+        </is>
+      </c>
+      <c r="G72" s="11" t="inlineStr"/>
+      <c r="H72" s="11" t="inlineStr"/>
+      <c r="I72" s="11" t="inlineStr"/>
+      <c r="J72" s="11" t="inlineStr"/>
+      <c r="K72" s="11" t="inlineStr"/>
+      <c r="L72" s="11" t="inlineStr"/>
+      <c r="M72" s="11" t="inlineStr">
+        <is>
           <t>Listed for retrieval</t>
         </is>
       </c>
-      <c r="N70" s="11" t="inlineStr">
+      <c r="N72" s="11" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="O70" s="11" t="inlineStr">
+      <c r="O72" s="11" t="inlineStr">
         <is>
           <t>NOT USED</t>
         </is>
       </c>
-      <c r="P70" s="11" t="inlineStr">
+      <c r="P72" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q70" s="11" t="inlineStr">
+      <c r="Q72" s="11" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R70" s="11" t="inlineStr"/>
-      <c r="S70" s="11" t="inlineStr"/>
-      <c r="T70" s="11" t="inlineStr">
+      <c r="R72" s="11" t="inlineStr"/>
+      <c r="S72" s="11" t="inlineStr"/>
+      <c r="T72" s="11" t="inlineStr">
         <is>
           <t>SR23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T70"/>
+  <autoFilter ref="A1:T72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7640,19 +7832,19 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>SR20</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>E3-01</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>PENDING PRIMARY DOCUMENT</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
         </is>
       </c>
     </row>

</xml_diff>